<commit_message>
Regenerar data validations netes a EXEMPLE i Plantilla
- Excel mostrava avís 'libro reparado' per validacions XML ambigües
- Recreades des de zero amb totes les propietats definides (title, prompt, error msg)
- Afecta tant l'EXEMPLE_Entrada_Mes_Demo.xlsx com la 02_Plantilla_Entrada.xlsx
</commit_message>
<xml_diff>
--- a/02_Plantilla_Entrada.xlsx
+++ b/02_Plantilla_Entrada.xlsx
@@ -1463,8 +1463,6 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="6" t="n"/>
     </row>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
@@ -1478,7 +1476,6 @@
           <t>rotador</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" s="12" t="inlineStr">
         <is>
           <t>Participa a la roda alfabètica de guàrdies. Cas habitual per a la majoria.</t>
@@ -1491,7 +1488,6 @@
           <t>fix-només</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" s="12" t="inlineStr">
         <is>
           <t>Només cobreix els seus torns fixos definits a Configuració. No participa a la roda.</t>
@@ -1504,7 +1500,6 @@
           <t>fix-i-rota</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" s="12" t="inlineStr">
         <is>
           <t>Té torns fixos però també participa a la roda per a guàrdies addicionals.</t>
@@ -1517,7 +1512,6 @@
           <t>sun-nit-only</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" s="12" t="inlineStr">
         <is>
           <t>Cas especial: només fa guàrdies de diumenge nit. Vegeu Configuració.</t>
@@ -1530,7 +1524,6 @@
           <t>weekend-day-only</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" s="12" t="inlineStr">
         <is>
           <t>Cas especial: només dissabte/diumenge dia. Vegeu Configuració.</t>
@@ -1543,7 +1536,6 @@
           <t>nou-incorporat</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" s="12" t="inlineStr">
         <is>
           <t>Nou professional en període de rodatge: només cobreix dimecres 16-20 (excepte 1r Dc del mes). Quan es consideri format, canvieu-li el rol a "rotador".</t>
@@ -1554,9 +1546,12 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="B4:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Valor no vàlid" promptTitle="Rol del professional" prompt="rotador = participa a la roda alfabètica&#10;fix-només = només cobreix torns fixos, no rota&#10;fix-i-rota = té torn fix però també participa a la roda&#10;sun-nit-only = només diumenge nit&#10;weekend-day-only = només dissabte/diumenge dia&#10;nou-incorporat = només dimecres 16-20 (excepte 1r del mes)" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="B4:B200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Rol no vàlid" error="Trieu una de les opcions del desplegable" promptTitle="Rol" prompt="Trieu el rol del professional" type="list">
       <formula1>"rotador,fix-només,fix-i-rota,sun-nit-only,weekend-day-only,nou-incorporat"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
v2.1: filtre Actiu (col. E), codi B=Baixa i marge de reincorporació de 3 dies
- load_input llegeix Radiòlegs!E i exclou els NO actius de la roda,
  dels nou-incorporats i dels perfils especials; els torns fixos
  d'un inactiu es marquen [SUBSTITUIR]
- nou codi B (Baixa) a la pestanya Vacances, idèntic a V
- DIES_REINCORPORACIO=3: després d'una absència V/B es bloquegen
  2 dies més; el professional no perd el torn
- validació, UI Streamlit, plantilles Excel i documentació al dia
- .gitignore: bloqueja plantilles i plannings amb dades reals
</commit_message>
<xml_diff>
--- a/02_Plantilla_Entrada.xlsx
+++ b/02_Plantilla_Entrada.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -661,40 +661,44 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   V = Vacances. No fa guàrdia aquell dia.</t>
+          <t xml:space="preserve">   V = Vacances. No fa guàrdia aquell dia + 2 dies de marge de reincorporació.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   C = Congrés. No fa guàrdia aquell dia.</t>
+          <t xml:space="preserve">   B = Baixa. Mateix comportament que V (bloqueja el dia + 2 dies de marge).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   G = Guàrdia en una altra institució. Bloqueja el dia, l'anterior i el posterior.</t>
+          <t xml:space="preserve">   C = Congrés. No fa guàrdia aquell dia (sense marge posterior).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   X = Guàrdia ja assignada (referència; no afecta l'algorisme).</t>
+          <t xml:space="preserve">   G = Guàrdia en una altra institució. Bloqueja el dia, l'anterior i el posterior.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">   X = Guàrdia ja assignada (referència; no afecta l'algorisme).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">   (buit) = Disponible.</t>
         </is>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
@@ -728,6 +732,71 @@
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Si hi ha diversos nou-incorporats, rotaran entre ells per als dimecres tarda. Quan es considerin formats, canvieu el rol a "rotador".</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ACTUALITZACIÓ: columna E "Actiu" de la pestanya Radiòlegs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Posa "No" a la columna E per treure un professional del planning NOMÉS aquest mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>NO cal esborrar la seva fila: queda fora de la roda, dels nou-incorporats i dels perfils especials,</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>i si té un torn fix assignat el planning hi escriurà [SUBSTITUIR]. El mes següent torna-ho a posar a "Sí".</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Deixar la cel·la buida equival a "Sí".</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ACTUALITZACIÓ: marge de reincorporació de 3 dies</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Quan una absència V o B s'acaba el dia D, el professional torna a entrar a la roda el dia D+3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Es bloquegen els dies D+1 i D+2 per donar-li temps a reincorporar-se.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>No perd el torn: es manté al davant de la cua fins que estigui disponible.</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1300,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1262,6 +1332,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Actiu aquest mes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n"/>
@@ -1463,6 +1538,8 @@
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="6" t="n"/>
     </row>
+    <row r="54"/>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
@@ -1547,10 +1624,10 @@
     <mergeCell ref="A1:C1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B4:B200" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Rol no vàlid" error="Trieu una de les opcions del desplegable" promptTitle="Rol" prompt="Trieu el rol del professional" type="list">
+    <dataValidation sqref="B4:B205" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Rol no vàlid" error="Tria un rol de la llista." promptTitle="Rol" prompt="rotador / fix-només / fix-i-rota / sun-nit-only / weekend-day-only / nou-incorporat" type="list">
       <formula1>"rotador,fix-només,fix-i-rota,sun-nit-only,weekend-day-only,nou-incorporat"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E200" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E4:E205" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Valor no vàlid" error="Només &quot;Sí&quot; o &quot;No&quot;." promptTitle="Actiu aquest mes" prompt="&quot;No&quot; = aquest mes no fa guàrdies (no cal esborrar la fila). Buit = Sí." type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4340,8 +4417,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B4:AF73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="V=vacances, C=congrés, G=guàrdia altre lloc, X=guàrdia assignada" type="list">
-      <formula1>"V,C,G,X"</formula1>
+    <dataValidation sqref="B4:AF75" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Codi no vàlid" error="Valors permesos: V (vacances), B (baixa), C (congrés), G (guàrdia externa), X (ja assignada)." promptTitle="Codi" prompt="V=vacances, B=baixa, C=congrés, G=guàrdia externa, X=ja assignada." type="list">
+      <formula1>"V,B,C,G,X"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>